<commit_message>
Adding test data for more access methods
</commit_message>
<xml_diff>
--- a/example-input-data/library-index.xlsx
+++ b/example-input-data/library-index.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MASTER" sheetId="1" r:id="R9476b5faf4454331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MASTER" sheetId="1" r:id="Ra667ed4374514baa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35,7 +35,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -57,6 +57,21 @@
         <x:fgColor rgb="FF005A70"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FBF9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF6FF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="10">
     <x:border/>
@@ -154,7 +169,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -217,6 +232,81 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -699,7 +789,7 @@
         <x:v>Keywords</x:v>
       </x:c>
       <x:c r="I6" s="18" t="str">
-        <x:v>Access_Rights</x:v>
+        <x:v>Access</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
         <x:v>PDF_file_name</x:v>
@@ -979,6 +1069,421 @@
       </x:c>
       <x:c r="Q11" s="25" t="str">
         <x:v>Example record only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="29" t="str">
+        <x:v>NQ-006</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="str">
+        <x:v>Incomplete inactive row - reef mangrove draft</x:v>
+      </x:c>
+      <x:c r="C12" s="30" t="str"/>
+      <x:c r="D12" s="30" t="str"/>
+      <x:c r="E12" s="30" t="str">
+        <x:v>Plant</x:v>
+      </x:c>
+      <x:c r="F12" s="30" t="str">
+        <x:v>Hinchinbrook</x:v>
+      </x:c>
+      <x:c r="G12" s="30" t="str"/>
+      <x:c r="H12" s="30" t="str">
+        <x:v>mangrove; estuary</x:v>
+      </x:c>
+      <x:c r="I12" s="30" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="J12" s="30" t="str"/>
+      <x:c r="K12" s="30" t="str"/>
+      <x:c r="L12" s="30" t="str">
+        <x:v>inactive</x:v>
+      </x:c>
+      <x:c r="M12" s="30" t="str"/>
+      <x:c r="N12" s="30" t="str"/>
+      <x:c r="O12" s="30" t="str"/>
+      <x:c r="P12" s="30" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q12" s="31" t="str">
+        <x:v>Deliberately incomplete inactive example row.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="32" t="str">
+        <x:v>NQ-007</x:v>
+      </x:c>
+      <x:c r="B13" s="33" t="str"/>
+      <x:c r="C13" s="33" t="str">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="D13" s="33" t="str"/>
+      <x:c r="E13" s="33" t="str">
+        <x:v>Reptile</x:v>
+      </x:c>
+      <x:c r="F13" s="33" t="str"/>
+      <x:c r="G13" s="33" t="str">
+        <x:v>Savanna woodland</x:v>
+      </x:c>
+      <x:c r="H13" s="33" t="str"/>
+      <x:c r="I13" s="33" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="J13" s="33" t="str">
+        <x:v>missing_inactive_example.pdf</x:v>
+      </x:c>
+      <x:c r="K13" s="33" t="str"/>
+      <x:c r="L13" s="33" t="str">
+        <x:v>inactive</x:v>
+      </x:c>
+      <x:c r="M13" s="33" t="str"/>
+      <x:c r="N13" s="33" t="str">
+        <x:v>Northern quoll skink placeholder</x:v>
+      </x:c>
+      <x:c r="O13" s="33" t="str"/>
+      <x:c r="P13" s="33" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q13" s="34" t="str">
+        <x:v>Deliberately incomplete inactive example row with a missing document.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="32" t="str">
+        <x:v>NQ-008</x:v>
+      </x:c>
+      <x:c r="B14" s="33" t="str">
+        <x:v>Incomplete inactive row - pandanus wetlands note</x:v>
+      </x:c>
+      <x:c r="C14" s="33" t="str"/>
+      <x:c r="D14" s="33" t="str">
+        <x:v>Wetlands Field Group</x:v>
+      </x:c>
+      <x:c r="E14" s="33" t="str"/>
+      <x:c r="F14" s="33" t="str">
+        <x:v>Atherton Tablelands</x:v>
+      </x:c>
+      <x:c r="G14" s="33" t="str"/>
+      <x:c r="H14" s="33" t="str">
+        <x:v>pandanus; wetland</x:v>
+      </x:c>
+      <x:c r="I14" s="33" t="str"/>
+      <x:c r="J14" s="33" t="str"/>
+      <x:c r="K14" s="33" t="str"/>
+      <x:c r="L14" s="33" t="str">
+        <x:v>inactive</x:v>
+      </x:c>
+      <x:c r="M14" s="33" t="str">
+        <x:v>Draft row retained to show inactive rows are excluded from processing.</x:v>
+      </x:c>
+      <x:c r="N14" s="33" t="str">
+        <x:v>Pandanus</x:v>
+      </x:c>
+      <x:c r="O14" s="33" t="str"/>
+      <x:c r="P14" s="33" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q14" s="34" t="str">
+        <x:v>Deliberately incomplete inactive example row with blank access rights.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A15" s="35" t="str">
+        <x:v>NQ-009</x:v>
+      </x:c>
+      <x:c r="B15" s="36" t="str">
+        <x:v>Golden bowerbird upland rainforest monitoring article</x:v>
+      </x:c>
+      <x:c r="C15" s="36" t="str">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="D15" s="36" t="str">
+        <x:v>Upland Rainforest Monitoring Team</x:v>
+      </x:c>
+      <x:c r="E15" s="36" t="str">
+        <x:v>Bird</x:v>
+      </x:c>
+      <x:c r="F15" s="36" t="str">
+        <x:v>Atherton Tablelands</x:v>
+      </x:c>
+      <x:c r="G15" s="36" t="str">
+        <x:v>Upland rainforest</x:v>
+      </x:c>
+      <x:c r="H15" s="36" t="str">
+        <x:v>golden bowerbird; upland rainforest; monitoring</x:v>
+      </x:c>
+      <x:c r="I15" s="36" t="str">
+        <x:v>download from publisher</x:v>
+      </x:c>
+      <x:c r="J15" s="36" t="str"/>
+      <x:c r="K15" s="36" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Golden_bowerbird</x:v>
+      </x:c>
+      <x:c r="L15" s="36" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="M15" s="36" t="str">
+        <x:v>Wikipedia summary: the golden bowerbird is a near-threatened bowerbird endemic to Queensland's Atherton region. It lives mainly in upland rainforest, and males build and decorate bowers as part of courtship.</x:v>
+      </x:c>
+      <x:c r="N15" s="36" t="str">
+        <x:v>Golden bowerbird</x:v>
+      </x:c>
+      <x:c r="O15" s="36" t="str">
+        <x:v>Near Threatened</x:v>
+      </x:c>
+      <x:c r="P15" s="36" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q15" s="37" t="str">
+        <x:v>Complete active publisher-access example row.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="35" t="str">
+        <x:v>NQ-010</x:v>
+      </x:c>
+      <x:c r="B16" s="36" t="str">
+        <x:v>Blue quandong seed dispersal in tropical restoration sites</x:v>
+      </x:c>
+      <x:c r="C16" s="36" t="str">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D16" s="36" t="str">
+        <x:v>Tropical Restoration Seed Ecology Group</x:v>
+      </x:c>
+      <x:c r="E16" s="36" t="str">
+        <x:v>Plant</x:v>
+      </x:c>
+      <x:c r="F16" s="36" t="str">
+        <x:v>Wet Tropics</x:v>
+      </x:c>
+      <x:c r="G16" s="36" t="str">
+        <x:v>Rainforest restoration plot</x:v>
+      </x:c>
+      <x:c r="H16" s="36" t="str">
+        <x:v>blue quandong; seed dispersal; restoration</x:v>
+      </x:c>
+      <x:c r="I16" s="36" t="str">
+        <x:v>download from publisher</x:v>
+      </x:c>
+      <x:c r="J16" s="36" t="str"/>
+      <x:c r="K16" s="36" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Elaeocarpus_grandis</x:v>
+      </x:c>
+      <x:c r="L16" s="36" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="M16" s="36" t="str">
+        <x:v>Wikipedia summary: Elaeocarpus grandis, commonly known as blue quandong, is a large buttressed rainforest tree native to coastal northeastern Australia. Its blue fruit is eaten by rainforest birds and mammals, and the species is associated with rainforest regeneration.</x:v>
+      </x:c>
+      <x:c r="N16" s="36" t="str">
+        <x:v>Blue quandong</x:v>
+      </x:c>
+      <x:c r="O16" s="36" t="str">
+        <x:v>Not listed</x:v>
+      </x:c>
+      <x:c r="P16" s="36" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q16" s="37" t="str">
+        <x:v>Complete active publisher-access example row.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A17" s="38" t="str">
+        <x:v>NQ-011</x:v>
+      </x:c>
+      <x:c r="B17" s="39" t="str">
+        <x:v>Northern bettong fire mosaic habitat brief</x:v>
+      </x:c>
+      <x:c r="C17" s="39" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="D17" s="39" t="str">
+        <x:v>Dry Tropics Mammal Research Group</x:v>
+      </x:c>
+      <x:c r="E17" s="39" t="str">
+        <x:v>Mammal</x:v>
+      </x:c>
+      <x:c r="F17" s="39" t="str">
+        <x:v>Mount Zero-Taravale</x:v>
+      </x:c>
+      <x:c r="G17" s="39" t="str">
+        <x:v>Open woodland; grassy understorey</x:v>
+      </x:c>
+      <x:c r="H17" s="39" t="str">
+        <x:v>northern bettong; fire mosaic; woodland</x:v>
+      </x:c>
+      <x:c r="I17" s="39" t="str">
+        <x:v>download from publisher</x:v>
+      </x:c>
+      <x:c r="J17" s="39" t="str"/>
+      <x:c r="K17" s="39" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Northern_bettong</x:v>
+      </x:c>
+      <x:c r="L17" s="39" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="M17" s="39" t="str">
+        <x:v>Wikipedia summary: the northern bettong is an endangered small marsupial from northeastern Australia. It is nocturnal, feeds mainly on fungi, roots and tubers, and is restricted to mixed open eucalypt and Allocasuarina forests near rainforest in far north Queensland.</x:v>
+      </x:c>
+      <x:c r="N17" s="39" t="str">
+        <x:v>Northern bettong</x:v>
+      </x:c>
+      <x:c r="O17" s="39" t="str">
+        <x:v>Endangered</x:v>
+      </x:c>
+      <x:c r="P17" s="39" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q17" s="40" t="str">
+        <x:v>Complete active publisher-access example row.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="42" t="str">
+        <x:v>NQ-012</x:v>
+      </x:c>
+      <x:c r="B18" s="43" t="str">
+        <x:v>Herbert River ringtail possum archival survey report</x:v>
+      </x:c>
+      <x:c r="C18" s="43" t="str">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="D18" s="43" t="str">
+        <x:v>Upland Mammal Survey Archive</x:v>
+      </x:c>
+      <x:c r="E18" s="43" t="str">
+        <x:v>Mammal</x:v>
+      </x:c>
+      <x:c r="F18" s="43" t="str">
+        <x:v>Herbert River Gorge</x:v>
+      </x:c>
+      <x:c r="G18" s="43" t="str">
+        <x:v>Upland rainforest; riparian corridor</x:v>
+      </x:c>
+      <x:c r="H18" s="43" t="str">
+        <x:v>Herbert River ringtail possum; archival survey; rainforest mammals</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="str">
+        <x:v>hardcopy</x:v>
+      </x:c>
+      <x:c r="J18" s="43" t="str"/>
+      <x:c r="K18" s="43" t="str"/>
+      <x:c r="L18" s="43" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="M18" s="43" t="str">
+        <x:v>Complete example record for a hardcopy-only survey report held offline and available by request.</x:v>
+      </x:c>
+      <x:c r="N18" s="43" t="str">
+        <x:v>Herbert River ringtail possum</x:v>
+      </x:c>
+      <x:c r="O18" s="43" t="str">
+        <x:v>Near Threatened</x:v>
+      </x:c>
+      <x:c r="P18" s="43" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q18" s="44" t="str">
+        <x:v>Hardcopy-only example; no file or publisher URL exists.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="45" t="str">
+        <x:v>NQ-013</x:v>
+      </x:c>
+      <x:c r="B19" s="46" t="str">
+        <x:v>Cape York cycads field herbarium notes</x:v>
+      </x:c>
+      <x:c r="C19" s="46" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="D19" s="46" t="str">
+        <x:v>Tropical Plant Collections Unit</x:v>
+      </x:c>
+      <x:c r="E19" s="46" t="str">
+        <x:v>Plant</x:v>
+      </x:c>
+      <x:c r="F19" s="46" t="str">
+        <x:v>Cape York Peninsula</x:v>
+      </x:c>
+      <x:c r="G19" s="46" t="str">
+        <x:v>Open woodland; sandstone outcrop</x:v>
+      </x:c>
+      <x:c r="H19" s="46" t="str">
+        <x:v>cycad; herbarium notes; Cape York flora</x:v>
+      </x:c>
+      <x:c r="I19" s="46" t="str">
+        <x:v>hardcopy</x:v>
+      </x:c>
+      <x:c r="J19" s="46" t="str"/>
+      <x:c r="K19" s="46" t="str"/>
+      <x:c r="L19" s="46" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="M19" s="46" t="str">
+        <x:v>Complete example record for hardcopy field notes that must be requested from the collection.</x:v>
+      </x:c>
+      <x:c r="N19" s="46" t="str">
+        <x:v>Cycad</x:v>
+      </x:c>
+      <x:c r="O19" s="46" t="str">
+        <x:v>Data Deficient</x:v>
+      </x:c>
+      <x:c r="P19" s="46" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q19" s="47" t="str">
+        <x:v>Hardcopy-only example; request access through the library contact pathway.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="48" t="str">
+        <x:v>NQ-014</x:v>
+      </x:c>
+      <x:c r="B20" s="49" t="str">
+        <x:v>Palm cockatoo nest tree assessment binder</x:v>
+      </x:c>
+      <x:c r="C20" s="49" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="D20" s="49" t="str">
+        <x:v>Cape York Woodland Research Group</x:v>
+      </x:c>
+      <x:c r="E20" s="49" t="str">
+        <x:v>Bird; Plant</x:v>
+      </x:c>
+      <x:c r="F20" s="49" t="str">
+        <x:v>Cape York Peninsula</x:v>
+      </x:c>
+      <x:c r="G20" s="49" t="str">
+        <x:v>Tropical savanna woodland; old-growth nesting trees</x:v>
+      </x:c>
+      <x:c r="H20" s="49" t="str">
+        <x:v>palm cockatoo; nest trees; savanna woodland</x:v>
+      </x:c>
+      <x:c r="I20" s="49" t="str">
+        <x:v>hardcopy</x:v>
+      </x:c>
+      <x:c r="J20" s="49" t="str"/>
+      <x:c r="K20" s="49" t="str"/>
+      <x:c r="L20" s="49" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="M20" s="49" t="str">
+        <x:v>Complete example record for an offline binder about nest-tree assessments and woodland habitat notes.</x:v>
+      </x:c>
+      <x:c r="N20" s="49" t="str">
+        <x:v>Palm cockatoo</x:v>
+      </x:c>
+      <x:c r="O20" s="49" t="str">
+        <x:v>Vulnerable</x:v>
+      </x:c>
+      <x:c r="P20" s="49" t="str">
+        <x:v>North Queensland Biodiversity Library</x:v>
+      </x:c>
+      <x:c r="Q20" s="50" t="str">
+        <x:v>Hardcopy-only example; not available online.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>